<commit_message>
Build: (6a8a902) Add brittle as effect
</commit_message>
<xml_diff>
--- a/cleanse.xlsx
+++ b/cleanse.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:B6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -406,18 +406,6 @@
       <c r="B1" t="str">
         <v>Effect</v>
       </c>
-      <c r="C1" t="str">
-        <v>Effect Amt</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Effect Hits</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Effect Dur</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Effect Target</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -426,12 +414,6 @@
       <c r="B2" t="str">
         <v>explode</v>
       </c>
-      <c r="C2" t="str">
-        <v>1</v>
-      </c>
-      <c r="E2" t="str">
-        <v>3</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -440,9 +422,6 @@
       <c r="B3" t="str">
         <v>charge</v>
       </c>
-      <c r="F3" t="str">
-        <v>self</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -451,12 +430,6 @@
       <c r="B4" t="str">
         <v>shield</v>
       </c>
-      <c r="C4" t="str">
-        <v>5</v>
-      </c>
-      <c r="F4" t="str">
-        <v>self</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -465,16 +438,18 @@
       <c r="B5" t="str">
         <v>freeze</v>
       </c>
-      <c r="C5" t="str">
-        <v>1</v>
-      </c>
-      <c r="E5" t="str">
-        <v>1</v>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Soul</v>
+      </c>
+      <c r="B6" t="str">
+        <v>energetic</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (f15007a) Add Enhance mode
</commit_message>
<xml_diff>
--- a/cleanse.xlsx
+++ b/cleanse.xlsx
@@ -398,6 +398,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="9" max="9" width="16.6640625" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="16.6640625" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" customWidth="1"/>
+    <col min="16" max="16" width="16.6640625" customWidth="1"/>
+    <col min="17" max="17" width="16.6640625" customWidth="1"/>
+    <col min="18" max="18" width="16.6640625" customWidth="1"/>
+    <col min="19" max="19" width="16.6640625" customWidth="1"/>
+    <col min="20" max="20" width="16.6640625" customWidth="1"/>
+    <col min="21" max="21" width="16.6640625" customWidth="1"/>
+    <col min="22" max="22" width="16.6640625" customWidth="1"/>
+    <col min="23" max="23" width="16.6640625" customWidth="1"/>
+    <col min="24" max="24" width="16.6640625" customWidth="1"/>
+    <col min="25" max="25" width="16.6640625" customWidth="1"/>
+    <col min="26" max="26" width="16.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,7 +440,7 @@
         <v>Fire</v>
       </c>
       <c r="B2" t="str">
-        <v>explode</v>
+        <v>combust</v>
       </c>
     </row>
     <row r="3">

</xml_diff>